<commit_message>
feat(F-NAR-019): TREE-AUT-017 polish Le citron dans le bol bleu
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-017.xlsx
+++ b/stories/arbres/TREE-AUT-017.xlsx
@@ -2766,17 +2766,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Le soleil du château n'a plus de sommet. J'ai le citron. On rentre. Le ballon reste contre le bac, oublié. Attends. Le jaune du parc n'est pas le nôtre. Le sac à étoiles pend à la barrière, trop haut. Je n'arrive pas au zip. Monte sur le bord. Mila ouvre. Une étoile de tissu brille. Elle glisse le manteau, le seau, le ballon. Le citron dessus, pour voir sa feuille. Merci. Tu as trouvé sa virgule dans le sable. Un grain rouge colle au sac bleu. Le bol nous attend.</t>
+          <t>Le soleil du château n'a plus de sommet. J'ai le citron. On rentre. Le ballon reste contre le bac, oublié. Attends. Le jaune du parc n'est pas le nôtre. Le sac à étoiles pend à la barrière, trop haut. Je n'arrive pas au zip. Monte sur le bord. Mila ouvre. Une étoile de tissu brille. Elle glisse le manteau, le seau, le ballon. Le citron dessus, pour voir sa feuille. Tu as trouvé sa virgule dans le sable. Un grain rouge colle au sac bleu. Le bol nous attend.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soleil du château n'a plus de sommet. J'ai le citron. On rentre. Le ballon reste contre le bac, oublié. Attends. Le jaune du parc n'est pas le nôtre. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière, trop haut. Je n'arrive pas au zip. Monte sur le bord. Mila ouvre. Une étoile de tissu brille. Elle glisse le manteau, le seau, le ballon. Le citron dessus, pour voir sa feuille. Merci. Tu as trouvé sa virgule dans le sable. Un grain rouge colle au sac bleu. Le bol nous attend.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soleil du château n'a plus de sommet. J'ai le citron. On rentre. Le ballon reste contre le bac, oublié. Attends. Le jaune du parc n'est pas le nôtre. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière, trop haut. Je n'arrive pas au zip. Monte sur le bord. Mila ouvre. Une étoile de tissu brille. Elle glisse le manteau, le seau, le ballon. Le citron dessus, pour voir sa feuille. Tu as trouvé sa virgule dans le sable. Un grain rouge colle au sac bleu. Le bol nous attend.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Le soleil du château n'a plus de sommet. J'ai le citron. On rentre. Le ballon reste contre le bac, oublié. Attends. Le jaune du parc n'est pas le nôtre. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière, trop haut. Je n'arrive pas au zip. Monte sur le bord. Mila ouvre. Une étoile de tissu brille. Elle glisse le manteau, le seau, le ballon. Le citron dessus, pour voir sa feuille. Merci. Tu as trouvé sa virgule dans le sable. Un grain rouge colle au sac bleu. Le bol nous attend. [pause]</t>
+          <t>Le soleil du château n'a plus de sommet. J'ai le citron. On rentre. Le ballon reste contre le bac, oublié. Attends. Le jaune du parc n'est pas le nôtre. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière, trop haut. Je n'arrive pas au zip. Monte sur le bord. Mila ouvre. Une étoile de tissu brille. Elle glisse le manteau, le seau, le ballon. Le citron dessus, pour voir sa feuille. Tu as trouvé sa virgule dans le sable. Un grain rouge colle au sac bleu. Le bol nous attend. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2923,7 +2923,6 @@
 narrateur|Une étoile de tissu brille.
 narrateur|Elle glisse le manteau, le seau, le ballon.
 enfant-f|Le citron dessus, pour voir sa feuille.
-papa|Merci.
 papa|Tu as trouvé sa virgule dans le sable.
 narrateur|Un grain rouge colle au sac bleu.
 enfant-f|Le bol nous attend.</t>
@@ -3146,17 +3145,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Le sable refroidit sous les paumes. Le ballon vient. Le citron aussi. Elle part. Le manteau reste plié sur le banc. Le banc n'est pas la maison, ma grande. Le sac à carreaux est ouvert sur le banc, large. Les carreaux aident à plier, un par un. Mila plie le manteau sur un carré rouge. Le seau entre. Le ballon entre. Le citron, tout seul, sur le dernier carré. Merci. Le sac à carreaux tient tout. Le ballon laisse une trace ronde au tissu. Le bol, au salon, a son rond à lui. On y va.</t>
+          <t>Le sable refroidit sous les paumes. Le ballon vient. Le citron aussi. Elle part. Le manteau reste plié sur le banc. Le banc n'est pas la maison, ma grande. Le sac à carreaux est ouvert sur le banc, large. Les carreaux aident à plier, un par un. Mila plie le manteau sur un carré rouge. Le seau entre. Le ballon entre. Le citron, tout seul, sur le dernier carré. Le sac à carreaux tient tout. Le ballon laisse une trace ronde au tissu. Le bol, au salon, a son rond à lui. On y va.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le sable refroidit sous les paumes. Le ballon vient. Le citron aussi. Elle part. Le manteau reste plié sur le banc. Le banc n'est pas la maison, ma grande. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est ouvert sur le banc, large. Les carreaux aident à plier, un par un. Mila plie le manteau sur un carré rouge. Le seau entre. Le ballon entre. Le citron, tout seul, sur le dernier carré. Merci. Le sac à carreaux tient tout. Le ballon laisse une trace ronde au tissu. Le bol, au salon, a son rond à lui. On y va.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le sable refroidit sous les paumes. Le ballon vient. Le citron aussi. Elle part. Le manteau reste plié sur le banc. Le banc n'est pas la maison, ma grande. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est ouvert sur le banc, large. Les carreaux aident à plier, un par un. Mila plie le manteau sur un carré rouge. Le seau entre. Le ballon entre. Le citron, tout seul, sur le dernier carré. Le sac à carreaux tient tout. Le ballon laisse une trace ronde au tissu. Le bol, au salon, a son rond à lui. On y va.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Le sable refroidit sous les paumes. Le ballon vient. Le citron aussi. Elle part. Le manteau reste plié sur le banc. Le banc n'est pas la maison, ma grande. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est ouvert sur le banc, large. Les carreaux aident à plier, un par un. Mila plie le manteau sur un carré rouge. Le seau entre. Le ballon entre. Le citron, tout seul, sur le dernier carré. Merci. Le sac à carreaux tient tout. Le ballon laisse une trace ronde au tissu. Le bol, au salon, a son rond à lui. On y va. [pause]</t>
+          <t>Le sable refroidit sous les paumes. Le ballon vient. Le citron aussi. Elle part. Le manteau reste plié sur le banc. Le banc n'est pas la maison, ma grande. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est ouvert sur le banc, large. Les carreaux aident à plier, un par un. Mila plie le manteau sur un carré rouge. Le seau entre. Le ballon entre. Le citron, tout seul, sur le dernier carré. Le sac à carreaux tient tout. Le ballon laisse une trace ronde au tissu. Le bol, au salon, a son rond à lui. On y va. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3302,7 +3301,6 @@
 narrateur|Le seau entre.
 narrateur|Le ballon entre.
 enfant-f|Le citron, tout seul, sur le dernier carré.
-maman|Merci.
 maman|Le sac à carreaux tient tout.
 narrateur|Le ballon laisse une trace ronde au tissu.
 papa|Le bol, au salon, a son rond à lui.
@@ -3528,17 +3526,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Un nuage passe sur le bac. Le château pâlit. Vite, le citron rentre. Elle serre le ballon. Le seau reste au bord. Le seau a chanté, tout à l'heure. Il vient. Le sac à ronds attend près de la grille. Un gros bouton de bois ferme la bouche. Ronds, comme le citron, comme le ballon. Tu comptes, puis tu glisses tout dedans. Manteau. Seau. Ballon. Citron. Merci. Tu as compté jusqu'au jaune. Un brin d'herbe reste au sac vert. La virgule a voyagé.</t>
+          <t>Un nuage passe sur le bac. Le château pâlit. Vite, le citron rentre. Elle serre le ballon. Le seau reste au bord. Le seau a chanté, tout à l'heure. Il vient. Le sac à ronds attend près de la grille. Un gros bouton de bois ferme la bouche. Ronds, comme le citron, comme le ballon. Tu comptes, puis tu glisses tout dedans. Manteau. Seau. Ballon. Citron. Tu as compté jusqu'au jaune. Un brin d'herbe reste au sac vert. La virgule a voyagé.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un nuage passe sur le bac. Le château pâlit. Vite, le citron rentre. Elle serre le ballon. Le seau reste au bord. Le seau a chanté, tout à l'heure. Il vient. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; attend près de la grille. Un gros bouton de bois ferme la bouche. Ronds, comme le citron, comme le ballon. Tu comptes, puis tu glisses tout dedans. Manteau. Seau. Ballon. Citron. Merci. Tu as compté jusqu'au jaune. Un brin d'herbe reste au sac vert. La virgule a voyagé.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un nuage passe sur le bac. Le château pâlit. Vite, le citron rentre. Elle serre le ballon. Le seau reste au bord. Le seau a chanté, tout à l'heure. Il vient. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; attend près de la grille. Un gros bouton de bois ferme la bouche. Ronds, comme le citron, comme le ballon. Tu comptes, puis tu glisses tout dedans. Manteau. Seau. Ballon. Citron. Tu as compté jusqu'au jaune. Un brin d'herbe reste au sac vert. La virgule a voyagé.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Un nuage passe sur le bac. Le château pâlit. Vite, le citron rentre. Elle serre le ballon. Le seau reste au bord. Le seau a chanté, tout à l'heure. Il vient. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; attend près de la grille. Un gros bouton de bois ferme la bouche. Ronds, comme le citron, comme le ballon. Tu comptes, puis tu glisses tout dedans. Manteau. Seau. Ballon. Citron. Merci. Tu as compté jusqu'au jaune. Un brin d'herbe reste au sac vert. La virgule a voyagé. [pause]</t>
+          <t>Un nuage passe sur le bac. Le château pâlit. Vite, le citron rentre. Elle serre le ballon. Le seau reste au bord. Le seau a chanté, tout à l'heure. Il vient. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; attend près de la grille. Un gros bouton de bois ferme la bouche. Ronds, comme le citron, comme le ballon. Tu comptes, puis tu glisses tout dedans. Manteau. Seau. Ballon. Citron. Tu as compté jusqu'au jaune. Un brin d'herbe reste au sac vert. La virgule a voyagé. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3687,7 +3685,6 @@
 narrateur|Seau.
 narrateur|Ballon.
 narrateur|Citron.
-papa|Merci.
 papa|Tu as compté jusqu'au jaune.
 narrateur|Un brin d'herbe reste au sac vert.
 enfant-f|La virgule a voyagé.</t>
@@ -4306,17 +4303,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Le seau est lourd. Le citron y fait clic. On rentre. J'ai tout. Le manteau, sur le banc, n'est pas dans le seau. Le clic du seau n'emporte pas le rouge. Le sac à étoiles pend. Mila tire le zip, crcr. L'anse d'abord, puis le tissu. Elle met le seau, le manteau, le citron au-dessus. Sa feuille, je la vois dans le zip. Merci. Le clic rentre avec nous. Du sable fin brille dans le sac bleu. Le bol, lui, n'a pas de sable. Le citron va le remplir. Une étoile de tissu garde un grain.</t>
+          <t>Le seau est lourd. Le citron y fait clic. On rentre. J'ai tout. Le manteau, sur le banc, n'est pas dans le seau. Le clic du seau n'emporte pas le rouge. Le sac à étoiles pend. Mila tire le zip, crcr. L'anse d'abord, puis le tissu. Elle met le seau, le manteau, le citron au-dessus. Sa feuille, je la vois dans le zip. Le clic rentre avec nous. Du sable fin brille dans le sac bleu. Le bol, lui, n'a pas de sable. Le citron va le remplir. Une étoile de tissu garde un grain.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau est lourd. Le citron y fait clic. On rentre. J'ai tout. Le manteau, sur le banc, n'est pas dans le seau. Le clic du seau n'emporte pas le rouge. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila tire le zip, crcr. L'anse d'abord, puis le tissu. Elle met le seau, le manteau, le citron au-dessus. Sa feuille, je la vois dans le zip. Merci. Le clic rentre avec nous. Du sable fin brille dans le sac bleu. Le bol, lui, n'a pas de sable. Le citron va le remplir. Une étoile de tissu garde un grain.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau est lourd. Le citron y fait clic. On rentre. J'ai tout. Le manteau, sur le banc, n'est pas dans le seau. Le clic du seau n'emporte pas le rouge. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila tire le zip, crcr. L'anse d'abord, puis le tissu. Elle met le seau, le manteau, le citron au-dessus. Sa feuille, je la vois dans le zip. Le clic rentre avec nous. Du sable fin brille dans le sac bleu. Le bol, lui, n'a pas de sable. Le citron va le remplir. Une étoile de tissu garde un grain.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Le seau est lourd. Le citron y fait clic. On rentre. J'ai tout. Le manteau, sur le banc, n'est pas dans le seau. Le clic du seau n'emporte pas le rouge. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila tire le zip, crcr. L'anse d'abord, puis le tissu. Elle met le seau, le manteau, le citron au-dessus. Sa feuille, je la vois dans le zip. Merci. Le clic rentre avec nous. Du sable fin brille dans le sac bleu. Le bol, lui, n'a pas de sable. Le citron va le remplir. Une étoile de tissu garde un grain. [pause]</t>
+          <t>Le seau est lourd. Le citron y fait clic. On rentre. J'ai tout. Le manteau, sur le banc, n'est pas dans le seau. Le clic du seau n'emporte pas le rouge. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila tire le zip, crcr. L'anse d'abord, puis le tissu. Elle met le seau, le manteau, le citron au-dessus. Sa feuille, je la vois dans le zip. Le clic rentre avec nous. Du sable fin brille dans le sac bleu. Le bol, lui, n'a pas de sable. Le citron va le remplir. Une étoile de tissu garde un grain. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4461,7 +4458,6 @@
 papa|L'anse d'abord, puis le tissu.
 narrateur|Elle met le seau, le manteau, le citron au-dessus.
 enfant-f|Sa feuille, je la vois dans le zip.
-papa|Merci.
 papa|Le clic rentre avec nous.
 narrateur|Du sable fin brille dans le sac bleu.
 maman|Le bol, lui, n'a pas de sable.
@@ -4687,17 +4683,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Mila veut partir le seau contre la hanche. Le citron est dedans. C'est bon. Le banc a ton manteau. Le bol n'a rien, lui. Le sac à carreaux est sur le banc, bouche ouverte. Un carreau pour le seau. Un carreau pour le rouge. Mila pose l'anse sur un carré, le manteau sur l'autre. Le citron, je le sors. Il va sur le bleu du sac. La virgule verte touche un carreau clair. Merci. Tu as sorti le soleil du sable. L'anse jaune touche le sac rouge. Au salon, le bol est bleu, pas rouge. Il va retrouver son bleu. Un grain reste au fond du seau, oublié.</t>
+          <t>Mila veut partir le seau contre la hanche. Le citron est dedans. C'est bon. Le banc a ton manteau. Le bol n'a rien, lui. Le sac à carreaux est sur le banc, bouche ouverte. Un carreau pour le seau. Un carreau pour le rouge. Mila pose l'anse sur un carré, le manteau sur l'autre. Le citron, je le sors. Il va sur le bleu du sac. La virgule verte touche un carreau clair. Tu as sorti le soleil du sable. L'anse jaune touche le sac rouge. Au salon, le bol est bleu, pas rouge. Il va retrouver son bleu. Un grain reste au fond du seau, oublié.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut partir le seau contre la hanche. Le citron est dedans. C'est bon. Le banc a ton manteau. Le bol n'a rien, lui. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, bouche ouverte. Un carreau pour le seau. Un carreau pour le rouge. Mila pose l'anse sur un carré, le manteau sur l'autre. Le citron, je le sors. Il va sur le bleu du sac. La virgule verte touche un carreau clair. Merci. Tu as sorti le soleil du sable. L'anse jaune touche le sac rouge. Au salon, le bol est bleu, pas rouge. Il va retrouver son bleu. Un grain reste au fond du seau, oublié.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut partir le seau contre la hanche. Le citron est dedans. C'est bon. Le banc a ton manteau. Le bol n'a rien, lui. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, bouche ouverte. Un carreau pour le seau. Un carreau pour le rouge. Mila pose l'anse sur un carré, le manteau sur l'autre. Le citron, je le sors. Il va sur le bleu du sac. La virgule verte touche un carreau clair. Tu as sorti le soleil du sable. L'anse jaune touche le sac rouge. Au salon, le bol est bleu, pas rouge. Il va retrouver son bleu. Un grain reste au fond du seau, oublié.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Mila veut partir le seau contre la hanche. Le citron est dedans. C'est bon. Le banc a ton manteau. Le bol n'a rien, lui. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, bouche ouverte. Un carreau pour le seau. Un carreau pour le rouge. Mila pose l'anse sur un carré, le manteau sur l'autre. Le citron, je le sors. Il va sur le bleu du sac. La virgule verte touche un carreau clair. Merci. Tu as sorti le soleil du sable. L'anse jaune touche le sac rouge. Au salon, le bol est bleu, pas rouge. Il va retrouver son bleu. Un grain reste au fond du seau, oublié. [pause]</t>
+          <t>Mila veut partir le seau contre la hanche. Le citron est dedans. C'est bon. Le banc a ton manteau. Le bol n'a rien, lui. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, bouche ouverte. Un carreau pour le seau. Un carreau pour le rouge. Mila pose l'anse sur un carré, le manteau sur l'autre. Le citron, je le sors. Il va sur le bleu du sac. La virgule verte touche un carreau clair. Tu as sorti le soleil du sable. L'anse jaune touche le sac rouge. Au salon, le bol est bleu, pas rouge. Il va retrouver son bleu. Un grain reste au fond du seau, oublié. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4843,7 +4839,6 @@
 enfant-f|Le citron, je le sors.
 enfant-f|Il va sur le bleu du sac.
 narrateur|La virgule verte touche un carreau clair.
-maman|Merci.
 maman|Tu as sorti le soleil du sable.
 narrateur|L'anse jaune touche le sac rouge.
 papa|Au salon, le bol est bleu, pas rouge.
@@ -5067,17 +5062,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau picore trop près du seau. Ce n'est pas à toi ! C'est mon soleil. Elle couvre le seau de sa main. L'oiseau s'en va. Le sac à ronds, près de la grille, est plus sûr. Le bouton de bois résiste. Mila le tourne. Seau, manteau, citron. Trois ronds. Elle glisse tout. Un coquillage minuscule roule au fond. Il était dans le sable. Merci. Tu as gardé le jaune pour le bol. Un coquillage minuscule roule au sac vert. Le bol n'a pas de coquillage. Je le lui rends. La virgule verte a un grain, et une poussière de coquille.</t>
+          <t>Un oiseau picore trop près du seau. Ce n'est pas à toi ! C'est mon soleil. Elle couvre le seau de sa main. L'oiseau s'en va. Le sac à ronds, près de la grille, est plus sûr. Le bouton de bois résiste. Mila le tourne. Seau, manteau, citron. Trois ronds. Elle glisse tout. Un coquillage minuscule roule au fond. Il était dans le sable. Tu as gardé le jaune pour le bol. Un coquillage minuscule roule au sac vert. Le bol n'a pas de coquillage. Je le lui rends. La virgule verte a un grain, et une poussière de coquille.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un oiseau picore trop près du seau. Ce n'est pas à toi ! C'est mon soleil. Elle couvre le seau de sa main. L'oiseau s'en va. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt;, près de la grille, est plus sûr. Le bouton de bois résiste. Mila le tourne. Seau, manteau, citron. Trois ronds. Elle glisse tout. Un coquillage minuscule roule au fond. Il était dans le sable. Merci. Tu as gardé le jaune pour le bol. Un coquillage minuscule roule au sac vert. Le bol n'a pas de coquillage. Je le lui rends. La virgule verte a un grain, et une poussière de coquille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un oiseau picore trop près du seau. Ce n'est pas à toi ! C'est mon soleil. Elle couvre le seau de sa main. L'oiseau s'en va. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt;, près de la grille, est plus sûr. Le bouton de bois résiste. Mila le tourne. Seau, manteau, citron. Trois ronds. Elle glisse tout. Un coquillage minuscule roule au fond. Il était dans le sable. Tu as gardé le jaune pour le bol. Un coquillage minuscule roule au sac vert. Le bol n'a pas de coquillage. Je le lui rends. La virgule verte a un grain, et une poussière de coquille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau picore trop près du seau. Ce n'est pas à toi ! C'est mon soleil. Elle couvre le seau de sa main. L'oiseau s'en va. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt;, près de la grille, est plus sûr. Le bouton de bois résiste. Mila le tourne. Seau, manteau, citron. Trois ronds. Elle glisse tout. Un coquillage minuscule roule au fond. Il était dans le sable. Merci. Tu as gardé le jaune pour le bol. Un coquillage minuscule roule au sac vert. Le bol n'a pas de coquillage. Je le lui rends. La virgule verte a un grain, et une poussière de coquille. [pause]</t>
+          <t>Un oiseau picore trop près du seau. Ce n'est pas à toi ! C'est mon soleil. Elle couvre le seau de sa main. L'oiseau s'en va. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt;, près de la grille, est plus sûr. Le bouton de bois résiste. Mila le tourne. Seau, manteau, citron. Trois ronds. Elle glisse tout. Un coquillage minuscule roule au fond. Il était dans le sable. Tu as gardé le jaune pour le bol. Un coquillage minuscule roule au sac vert. Le bol n'a pas de coquillage. Je le lui rends. La virgule verte a un grain, et une poussière de coquille. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5224,7 +5219,6 @@
 narrateur|Elle glisse tout.
 narrateur|Un coquillage minuscule roule au fond.
 enfant-f|Il était dans le sable.
-papa|Merci.
 papa|Tu as gardé le jaune pour le bol.
 narrateur|Un coquillage minuscule roule au sac vert.
 maman|Le bol n'a pas de coquillage.
@@ -5845,17 +5839,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a l'oreille pleine de sable. On rentre, toi et le soleil. Le seau reste au bord. Le manteau aussi. Le gris n'emporte pas le jaune du seau. Le sac à étoiles pend. Mila saute un peu. Zip. Doudou d'abord, tête vers le haut. L'oreille dépasse. Puis le manteau. Puis le seau. Le citron contre l'oreille, pour qu'il n'ait pas froid. Merci. Tu as sorti le sable de l'oreille, aussi. Le bol va voir un soleil un peu tiède. Il a dormi contre le doudou. Un fil gris pend, pris dans le zip.</t>
+          <t>Le doudou a l'oreille pleine de sable. On rentre, toi et le soleil. Le seau reste au bord. Le manteau aussi. Le gris n'emporte pas le jaune du seau. Le sac à étoiles pend. Mila saute un peu. Zip. Doudou d'abord, tête vers le haut. L'oreille dépasse. Puis le manteau. Puis le seau. Le citron contre l'oreille, pour qu'il n'ait pas froid. Tu as sorti le sable de l'oreille, aussi. Le bol va voir un soleil un peu tiède. Il a dormi contre le doudou. Un fil gris pend, pris dans le zip.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou a l'oreille pleine de sable. On rentre, toi et le soleil. Le seau reste au bord. Le manteau aussi. Le gris n'emporte pas le jaune du seau. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila saute un peu. Zip. Doudou d'abord, tête vers le haut. L'oreille dépasse. Puis le manteau. Puis le seau. Le citron contre l'oreille, pour qu'il n'ait pas froid. Merci. Tu as sorti le sable de l'oreille, aussi. Le bol va voir un soleil un peu tiède. Il a dormi contre le doudou. Un fil gris pend, pris dans le zip.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou a l'oreille pleine de sable. On rentre, toi et le soleil. Le seau reste au bord. Le manteau aussi. Le gris n'emporte pas le jaune du seau. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila saute un peu. Zip. Doudou d'abord, tête vers le haut. L'oreille dépasse. Puis le manteau. Puis le seau. Le citron contre l'oreille, pour qu'il n'ait pas froid. Tu as sorti le sable de l'oreille, aussi. Le bol va voir un soleil un peu tiède. Il a dormi contre le doudou. Un fil gris pend, pris dans le zip.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a l'oreille pleine de sable. On rentre, toi et le soleil. Le seau reste au bord. Le manteau aussi. Le gris n'emporte pas le jaune du seau. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila saute un peu. Zip. Doudou d'abord, tête vers le haut. L'oreille dépasse. Puis le manteau. Puis le seau. Le citron contre l'oreille, pour qu'il n'ait pas froid. Merci. Tu as sorti le sable de l'oreille, aussi. Le bol va voir un soleil un peu tiède. Il a dormi contre le doudou. Un fil gris pend, pris dans le zip. [pause]</t>
+          <t>Le doudou a l'oreille pleine de sable. On rentre, toi et le soleil. Le seau reste au bord. Le manteau aussi. Le gris n'emporte pas le jaune du seau. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila saute un peu. Zip. Doudou d'abord, tête vers le haut. L'oreille dépasse. Puis le manteau. Puis le seau. Le citron contre l'oreille, pour qu'il n'ait pas froid. Tu as sorti le sable de l'oreille, aussi. Le bol va voir un soleil un peu tiède. Il a dormi contre le doudou. Un fil gris pend, pris dans le zip. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -6002,7 +5996,6 @@
 narrateur|Puis le manteau.
 narrateur|Puis le seau.
 enfant-f|Le citron contre l'oreille, pour qu'il n'ait pas froid.
-papa|Merci.
 papa|Tu as sorti le sable de l'oreille, aussi.
 maman|Le bol va voir un soleil un peu tiède.
 enfant-f|Il a dormi contre le doudou.
@@ -6226,17 +6219,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Mila serre le doudou. Le citron est contre le gris. On a fini le château. Le banc a le manteau. Le bord a le seau. Le sac à carreaux attend, plié en deux sur le banc. Un carreau gris, un carreau rouge, un carreau jaune. Doudou. Manteau. Seau. Puis le citron au milieu. Il est au centre, comme au château. Merci. Tu as remis le soleil au milieu. Le doudou sent le sable, contre le sac rouge. Au salon, le bol est le milieu, lui. J'y pense. Un fil de laine du doudou reste au carreau.</t>
+          <t>Mila serre le doudou. Le citron est contre le gris. On a fini le château. Le banc a le manteau. Le bord a le seau. Le sac à carreaux attend, plié en deux sur le banc. Un carreau gris, un carreau rouge, un carreau jaune. Doudou. Manteau. Seau. Puis le citron au milieu. Il est au centre, comme au château. Tu as remis le soleil au milieu. Le doudou sent le sable, contre le sac rouge. Au salon, le bol est le milieu, lui. J'y pense. Un fil de laine du doudou reste au carreau.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila serre le doudou. Le citron est contre le gris. On a fini le château. Le banc a le manteau. Le bord a le seau. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; attend, plié en deux sur le banc. Un carreau gris, un carreau rouge, un carreau jaune. Doudou. Manteau. Seau. Puis le citron au milieu. Il est au centre, comme au château. Merci. Tu as remis le soleil au milieu. Le doudou sent le sable, contre le sac rouge. Au salon, le bol est le milieu, lui. J'y pense. Un fil de laine du doudou reste au carreau.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila serre le doudou. Le citron est contre le gris. On a fini le château. Le banc a le manteau. Le bord a le seau. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; attend, plié en deux sur le banc. Un carreau gris, un carreau rouge, un carreau jaune. Doudou. Manteau. Seau. Puis le citron au milieu. Il est au centre, comme au château. Tu as remis le soleil au milieu. Le doudou sent le sable, contre le sac rouge. Au salon, le bol est le milieu, lui. J'y pense. Un fil de laine du doudou reste au carreau.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Mila serre le doudou. Le citron est contre le gris. On a fini le château. Le banc a le manteau. Le bord a le seau. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; attend, plié en deux sur le banc. Un carreau gris, un carreau rouge, un carreau jaune. Doudou. Manteau. Seau. Puis le citron au milieu. Il est au centre, comme au château. Merci. Tu as remis le soleil au milieu. Le doudou sent le sable, contre le sac rouge. Au salon, le bol est le milieu, lui. J'y pense. Un fil de laine du doudou reste au carreau. [pause]</t>
+          <t>Mila serre le doudou. Le citron est contre le gris. On a fini le château. Le banc a le manteau. Le bord a le seau. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; attend, plié en deux sur le banc. Un carreau gris, un carreau rouge, un carreau jaune. Doudou. Manteau. Seau. Puis le citron au milieu. Il est au centre, comme au château. Tu as remis le soleil au milieu. Le doudou sent le sable, contre le sac rouge. Au salon, le bol est le milieu, lui. J'y pense. Un fil de laine du doudou reste au carreau. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6382,7 +6375,6 @@
 narrateur|Seau.
 narrateur|Puis le citron au milieu.
 enfant-f|Il est au centre, comme au château.
-maman|Merci.
 maman|Tu as remis le soleil au milieu.
 narrateur|Le doudou sent le sable, contre le sac rouge.
 papa|Au salon, le bol est le milieu, lui.
@@ -6610,17 +6602,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Un vent lève un peu de sable. Le doudou cligne. On part, avant qu'il ait trop de grains. La grille. Le sac à ronds a un bouton, pas de sable. Mila tourne le bouton. Ça résiste, puis ça cède. Rond le doudou, rond le seau, rond le citron. Elle glisse le manteau en dernier, comme un toit. Le toit du château, pour rentrer. Merci. Tu as fermé le bouton, toute seule. Un fil gris pend du sac vert. Le bol n'a pas de toit. Il a un rond de lumière. Je lui rends son soleil. La virgule verte a un grain, pris dans le fil.</t>
+          <t>Un vent lève un peu de sable. Le doudou cligne. On part, avant qu'il ait trop de grains. La grille. Le sac à ronds a un bouton, pas de sable. Mila tourne le bouton. Ça résiste, puis ça cède. Rond le doudou, rond le seau, rond le citron. Elle glisse le manteau en dernier, comme un toit. Le toit du château, pour rentrer. Tu as fermé le bouton, toute seule. Un fil gris pend du sac vert. Le bol n'a pas de toit. Il a un rond de lumière. Je lui rends son soleil. La virgule verte a un grain, pris dans le fil.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un vent lève un peu de sable. Le doudou cligne. On part, avant qu'il ait trop de grains. La grille. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; a un bouton, pas de sable. Mila tourne le bouton. Ça résiste, puis ça cède. Rond le doudou, rond le seau, rond le citron. Elle glisse le manteau en dernier, comme un toit. Le toit du château, pour rentrer. Merci. Tu as fermé le bouton, toute seule. Un fil gris pend du sac vert. Le bol n'a pas de toit. Il a un rond de lumière. Je lui rends son soleil. La virgule verte a un grain, pris dans le fil.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un vent lève un peu de sable. Le doudou cligne. On part, avant qu'il ait trop de grains. La grille. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; a un bouton, pas de sable. Mila tourne le bouton. Ça résiste, puis ça cède. Rond le doudou, rond le seau, rond le citron. Elle glisse le manteau en dernier, comme un toit. Le toit du château, pour rentrer. Tu as fermé le bouton, toute seule. Un fil gris pend du sac vert. Le bol n'a pas de toit. Il a un rond de lumière. Je lui rends son soleil. La virgule verte a un grain, pris dans le fil.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Un vent lève un peu de sable. Le doudou cligne. On part, avant qu'il ait trop de grains. La grille. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; a un bouton, pas de sable. Mila tourne le bouton. Ça résiste, puis ça cède. Rond le doudou, rond le seau, rond le citron. Elle glisse le manteau en dernier, comme un toit. Le toit du château, pour rentrer. Merci. Tu as fermé le bouton, toute seule. Un fil gris pend du sac vert. Le bol n'a pas de toit. Il a un rond de lumière. Je lui rends son soleil. La virgule verte a un grain, pris dans le fil. [pause]</t>
+          <t>Un vent lève un peu de sable. Le doudou cligne. On part, avant qu'il ait trop de grains. La grille. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; a un bouton, pas de sable. Mila tourne le bouton. Ça résiste, puis ça cède. Rond le doudou, rond le seau, rond le citron. Elle glisse le manteau en dernier, comme un toit. Le toit du château, pour rentrer. Tu as fermé le bouton, toute seule. Un fil gris pend du sac vert. Le bol n'a pas de toit. Il a un rond de lumière. Je lui rends son soleil. La virgule verte a un grain, pris dans le fil. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6764,7 +6756,6 @@
 maman|Rond le doudou, rond le seau, rond le citron.
 narrateur|Elle glisse le manteau en dernier, comme un toit.
 enfant-f|Le toit du château, pour rentrer.
-papa|Merci.
 papa|Tu as fermé le bouton, toute seule.
 narrateur|Un fil gris pend du sac vert.
 maman|Le bol n'a pas de toit.
@@ -8149,17 +8140,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>La rampe du toboggan se tait. Le ballon et le citron, je les ai. Le seau, près des marches, n'a pas bougé. Le ballon n'emporte pas l'anse. Le sac à étoiles pend à la barrière du toboggan. Le zip, j'y arrive, cette fois. Elle ouvre. Une étoile, puis le manteau, le seau, le ballon. Le citron au-dessus. Sa feuille a vu la rampe. Merci. Tu l'as sorti de sous le métal. La feuille jaune de la rampe colle au sac bleu. C'est sa médaille. Le bol préférera le zeste à la médaille. Le ballon s'enfonce, un peu froid.</t>
+          <t>La rampe du toboggan se tait. Le ballon et le citron, je les ai. Le seau, près des marches, n'a pas bougé. Le ballon n'emporte pas l'anse. Le sac à étoiles pend à la barrière du toboggan. Le zip, j'y arrive, cette fois. Elle ouvre. Une étoile, puis le manteau, le seau, le ballon. Le citron au-dessus. Sa feuille a vu la rampe. Tu l'as sorti de sous le métal. La feuille jaune de la rampe colle au sac bleu. C'est sa médaille. Le bol préférera le zeste à la médaille. Le ballon s'enfonce, un peu froid.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La rampe du toboggan se tait. Le ballon et le citron, je les ai. Le seau, près des marches, n'a pas bougé. Le ballon n'emporte pas l'anse. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière du toboggan. Le zip, j'y arrive, cette fois. Elle ouvre. Une étoile, puis le manteau, le seau, le ballon. Le citron au-dessus. Sa feuille a vu la rampe. Merci. Tu l'as sorti de sous le métal. La feuille jaune de la rampe colle au sac bleu. C'est sa médaille. Le bol préférera le zeste à la médaille. Le ballon s'enfonce, un peu froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La rampe du toboggan se tait. Le ballon et le citron, je les ai. Le seau, près des marches, n'a pas bougé. Le ballon n'emporte pas l'anse. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière du toboggan. Le zip, j'y arrive, cette fois. Elle ouvre. Une étoile, puis le manteau, le seau, le ballon. Le citron au-dessus. Sa feuille a vu la rampe. Tu l'as sorti de sous le métal. La feuille jaune de la rampe colle au sac bleu. C'est sa médaille. Le bol préférera le zeste à la médaille. Le ballon s'enfonce, un peu froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>La rampe du toboggan se tait. Le ballon et le citron, je les ai. Le seau, près des marches, n'a pas bougé. Le ballon n'emporte pas l'anse. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière du toboggan. Le zip, j'y arrive, cette fois. Elle ouvre. Une étoile, puis le manteau, le seau, le ballon. Le citron au-dessus. Sa feuille a vu la rampe. Merci. Tu l'as sorti de sous le métal. La feuille jaune de la rampe colle au sac bleu. C'est sa médaille. Le bol préférera le zeste à la médaille. Le ballon s'enfonce, un peu froid. [pause]</t>
+          <t>La rampe du toboggan se tait. Le ballon et le citron, je les ai. Le seau, près des marches, n'a pas bougé. Le ballon n'emporte pas l'anse. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière du toboggan. Le zip, j'y arrive, cette fois. Elle ouvre. Une étoile, puis le manteau, le seau, le ballon. Le citron au-dessus. Sa feuille a vu la rampe. Tu l'as sorti de sous le métal. La feuille jaune de la rampe colle au sac bleu. C'est sa médaille. Le bol préférera le zeste à la médaille. Le ballon s'enfonce, un peu froid. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8303,7 +8294,6 @@
 narrateur|Une étoile, puis le manteau, le seau, le ballon.
 maman|Le citron au-dessus.
 maman|Sa feuille a vu la rampe.
-papa|Merci.
 papa|Tu l'as sorti de sous le métal.
 narrateur|La feuille jaune de la rampe colle au sac bleu.
 enfant-f|C'est sa médaille.
@@ -8531,17 +8521,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Le ballon est un peu froid, près de la rampe. On rentre. J'ai mon soleil. Le banc a le manteau. Les marches ont le seau. Le sac à carreaux est posé sur le banc du toboggan. Carré pour le ballon. Carré pour le seau. Mila range. Le citron, elle le garde au creux de la main. Toi, tu ne glisses plus. Tu rentres. Merci. Tu as gardé le jaune hors de la rampe. Le ballon est un peu froid, près du sac rouge. Au salon, le bol est tiède, lui. Il va le réchauffer. Une feuille de rampe sèche au bord du sac.</t>
+          <t>Le ballon est un peu froid, près de la rampe. On rentre. J'ai mon soleil. Le banc a le manteau. Les marches ont le seau. Le sac à carreaux est posé sur le banc du toboggan. Carré pour le ballon. Carré pour le seau. Mila range. Le citron, elle le garde au creux de la main. Toi, tu ne glisses plus. Tu rentres. Tu as gardé le jaune hors de la rampe. Le ballon est un peu froid, près du sac rouge. Au salon, le bol est tiède, lui. Il va le réchauffer. Une feuille de rampe sèche au bord du sac.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon est un peu froid, près de la rampe. On rentre. J'ai mon soleil. Le banc a le manteau. Les marches ont le seau. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est posé sur le banc du toboggan. Carré pour le ballon. Carré pour le seau. Mila range. Le citron, elle le garde au creux de la main. Toi, tu ne glisses plus. Tu rentres. Merci. Tu as gardé le jaune hors de la rampe. Le ballon est un peu froid, près du sac rouge. Au salon, le bol est tiède, lui. Il va le réchauffer. Une feuille de rampe sèche au bord du sac.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon est un peu froid, près de la rampe. On rentre. J'ai mon soleil. Le banc a le manteau. Les marches ont le seau. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est posé sur le banc du toboggan. Carré pour le ballon. Carré pour le seau. Mila range. Le citron, elle le garde au creux de la main. Toi, tu ne glisses plus. Tu rentres. Tu as gardé le jaune hors de la rampe. Le ballon est un peu froid, près du sac rouge. Au salon, le bol est tiède, lui. Il va le réchauffer. Une feuille de rampe sèche au bord du sac.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Le ballon est un peu froid, près de la rampe. On rentre. J'ai mon soleil. Le banc a le manteau. Les marches ont le seau. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est posé sur le banc du toboggan. Carré pour le ballon. Carré pour le seau. Mila range. Le citron, elle le garde au creux de la main. Toi, tu ne glisses plus. Tu rentres. Merci. Tu as gardé le jaune hors de la rampe. Le ballon est un peu froid, près du sac rouge. Au salon, le bol est tiède, lui. Il va le réchauffer. Une feuille de rampe sèche au bord du sac. [pause]</t>
+          <t>Le ballon est un peu froid, près de la rampe. On rentre. J'ai mon soleil. Le banc a le manteau. Les marches ont le seau. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est posé sur le banc du toboggan. Carré pour le ballon. Carré pour le seau. Mila range. Le citron, elle le garde au creux de la main. Toi, tu ne glisses plus. Tu rentres. Tu as gardé le jaune hors de la rampe. Le ballon est un peu froid, près du sac rouge. Au salon, le bol est tiède, lui. Il va le réchauffer. Une feuille de rampe sèche au bord du sac. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8687,7 +8677,6 @@
 narrateur|Le citron, elle le garde au creux de la main.
 enfant-f|Toi, tu ne glisses plus.
 enfant-f|Tu rentres.
-maman|Merci.
 maman|Tu as gardé le jaune hors de la rampe.
 narrateur|Le ballon est un peu froid, près du sac rouge.
 papa|Au salon, le bol est tiède, lui.
@@ -8915,17 +8904,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe de la rampe, lente. Le ballon va rentrer, avant d'être mouillé. Le seau, les marches, le manteau. Avec nous. Le sac à ronds est près de la grille du toboggan. Le bouton de bois est humide. Mila le tourne. Ronds : ballon, citron, bouton. Elle glisse le seau, le manteau, le ballon. Le citron au milieu, au sec. Merci. Tu l'as sorti de la goutte. Une goutte glisse vers le sac vert, puis s'arrête. Le bol, au salon, n'a pas de goutte. Que du clic. La virgule verte a une perle d'eau, minuscule.</t>
+          <t>Une goutte tombe de la rampe, lente. Le ballon va rentrer, avant d'être mouillé. Le seau, les marches, le manteau. Avec nous. Le sac à ronds est près de la grille du toboggan. Le bouton de bois est humide. Mila le tourne. Ronds : ballon, citron, bouton. Elle glisse le seau, le manteau, le ballon. Le citron au milieu, au sec. Tu l'as sorti de la goutte. Une goutte glisse vers le sac vert, puis s'arrête. Le bol, au salon, n'a pas de goutte. Que du clic. La virgule verte a une perle d'eau, minuscule.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte tombe de la rampe, lente. Le ballon va rentrer, avant d'être mouillé. Le seau, les marches, le manteau. Avec nous. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; est près de la grille du toboggan. Le bouton de bois est humide. Mila le tourne. Ronds : ballon, citron, bouton. Elle glisse le seau, le manteau, le ballon. Le citron au milieu, au sec. Merci. Tu l'as sorti de la goutte. Une goutte glisse vers le sac vert, puis s'arrête. Le bol, au salon, n'a pas de goutte. Que du clic. La virgule verte a une perle d'eau, minuscule.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte tombe de la rampe, lente. Le ballon va rentrer, avant d'être mouillé. Le seau, les marches, le manteau. Avec nous. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; est près de la grille du toboggan. Le bouton de bois est humide. Mila le tourne. Ronds : ballon, citron, bouton. Elle glisse le seau, le manteau, le ballon. Le citron au milieu, au sec. Tu l'as sorti de la goutte. Une goutte glisse vers le sac vert, puis s'arrête. Le bol, au salon, n'a pas de goutte. Que du clic. La virgule verte a une perle d'eau, minuscule.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe de la rampe, lente. Le ballon va rentrer, avant d'être mouillé. Le seau, les marches, le manteau. Avec nous. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; est près de la grille du toboggan. Le bouton de bois est humide. Mila le tourne. Ronds : ballon, citron, bouton. Elle glisse le seau, le manteau, le ballon. Le citron au milieu, au sec. Merci. Tu l'as sorti de la goutte. Une goutte glisse vers le sac vert, puis s'arrête. Le bol, au salon, n'a pas de goutte. Que du clic. La virgule verte a une perle d'eau, minuscule. [pause]</t>
+          <t>Une goutte tombe de la rampe, lente. Le ballon va rentrer, avant d'être mouillé. Le seau, les marches, le manteau. Avec nous. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; est près de la grille du toboggan. Le bouton de bois est humide. Mila le tourne. Ronds : ballon, citron, bouton. Elle glisse le seau, le manteau, le ballon. Le citron au milieu, au sec. Tu l'as sorti de la goutte. Une goutte glisse vers le sac vert, puis s'arrête. Le bol, au salon, n'a pas de goutte. Que du clic. La virgule verte a une perle d'eau, minuscule. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -9069,7 +9058,6 @@
 maman|Ronds : ballon, citron, bouton.
 narrateur|Elle glisse le seau, le manteau, le ballon.
 enfant-f|Le citron au milieu, au sec.
-papa|Merci.
 papa|Tu l'as sorti de la goutte.
 narrateur|Une goutte glisse vers le sac vert, puis s'arrête.
 maman|Le bol, au salon, n'a pas de goutte.
@@ -9688,17 +9676,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Le seau a sonné contre les marches, toute la descente. On a fini de glisser. Le manteau, sur le banc, n'a pas sonné. Il vient, lui aussi, sans musique. Le sac à étoiles pend. Mila tire, crcr. Le seau droit, comme sur les marches. Elle le pose, anse vers le zip, pour le tenir. Le citron au-dessus. Plus de pente. Merci. Tes deux mains ont tenu l'anse. Le seau sonne, très bas, contre le sac bleu. Au salon, le bol n'a pas de pente. Il est plat. Il attend. Une étoile de tissu a un choc de plastique.</t>
+          <t>Le seau a sonné contre les marches, toute la descente. On a fini de glisser. Le manteau, sur le banc, n'a pas sonné. Il vient, lui aussi, sans musique. Le sac à étoiles pend. Mila tire, crcr. Le seau droit, comme sur les marches. Elle le pose, anse vers le zip, pour le tenir. Le citron au-dessus. Plus de pente. Tes deux mains ont tenu l'anse. Le seau sonne, très bas, contre le sac bleu. Au salon, le bol n'a pas de pente. Il est plat. Il attend. Une étoile de tissu a un choc de plastique.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau a sonné contre les marches, toute la descente. On a fini de glisser. Le manteau, sur le banc, n'a pas sonné. Il vient, lui aussi, sans musique. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila tire, crcr. Le seau droit, comme sur les marches. Elle le pose, anse vers le zip, pour le tenir. Le citron au-dessus. Plus de pente. Merci. Tes deux mains ont tenu l'anse. Le seau sonne, très bas, contre le sac bleu. Au salon, le bol n'a pas de pente. Il est plat. Il attend. Une étoile de tissu a un choc de plastique.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau a sonné contre les marches, toute la descente. On a fini de glisser. Le manteau, sur le banc, n'a pas sonné. Il vient, lui aussi, sans musique. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila tire, crcr. Le seau droit, comme sur les marches. Elle le pose, anse vers le zip, pour le tenir. Le citron au-dessus. Plus de pente. Tes deux mains ont tenu l'anse. Le seau sonne, très bas, contre le sac bleu. Au salon, le bol n'a pas de pente. Il est plat. Il attend. Une étoile de tissu a un choc de plastique.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Le seau a sonné contre les marches, toute la descente. On a fini de glisser. Le manteau, sur le banc, n'a pas sonné. Il vient, lui aussi, sans musique. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila tire, crcr. Le seau droit, comme sur les marches. Elle le pose, anse vers le zip, pour le tenir. Le citron au-dessus. Plus de pente. Merci. Tes deux mains ont tenu l'anse. Le seau sonne, très bas, contre le sac bleu. Au salon, le bol n'a pas de pente. Il est plat. Il attend. Une étoile de tissu a un choc de plastique. [pause]</t>
+          <t>Le seau a sonné contre les marches, toute la descente. On a fini de glisser. Le manteau, sur le banc, n'a pas sonné. Il vient, lui aussi, sans musique. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila tire, crcr. Le seau droit, comme sur les marches. Elle le pose, anse vers le zip, pour le tenir. Le citron au-dessus. Plus de pente. Tes deux mains ont tenu l'anse. Le seau sonne, très bas, contre le sac bleu. Au salon, le bol n'a pas de pente. Il est plat. Il attend. Une étoile de tissu a un choc de plastique. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9842,7 +9830,6 @@
 narrateur|Elle le pose, anse vers le zip, pour le tenir.
 enfant-f|Le citron au-dessus.
 enfant-f|Plus de pente.
-papa|Merci.
 papa|Tes deux mains ont tenu l'anse.
 narrateur|Le seau sonne, très bas, contre le sac bleu.
 maman|Au salon, le bol n'a pas de pente.
@@ -10071,17 +10058,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Le métal du toboggan se tait, près du banc. Le seau rentre. Le citron aussi. Le manteau, sur le banc, n'est pas une marche. Le sac à carreaux est ouvert, comme une rampe douce. On glisse les affaires, sans les jeter. Mila glisse le seau, puis le manteau, puis le citron. Une glissade sage, celle-là. Merci. Tu as choisi la pente du sac. Le métal du toboggan se tait, près du sac rouge. Le bol, lui, n'est pas une rampe. Je le sais. Je le remplis. Un carreau garde une trace d'anse.</t>
+          <t>Le métal du toboggan se tait, près du banc. Le seau rentre. Le citron aussi. Le manteau, sur le banc, n'est pas une marche. Le sac à carreaux est ouvert, comme une rampe douce. On glisse les affaires, sans les jeter. Mila glisse le seau, puis le manteau, puis le citron. Une glissade sage, celle-là. Tu as choisi la pente du sac. Le métal du toboggan se tait, près du sac rouge. Le bol, lui, n'est pas une rampe. Je le sais. Je le remplis. Un carreau garde une trace d'anse.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le métal du toboggan se tait, près du banc. Le seau rentre. Le citron aussi. Le manteau, sur le banc, n'est pas une marche. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est ouvert, comme une rampe douce. On glisse les affaires, sans les jeter. Mila glisse le seau, puis le manteau, puis le citron. Une glissade sage, celle-là. Merci. Tu as choisi la pente du sac. Le métal du toboggan se tait, près du sac rouge. Le bol, lui, n'est pas une rampe. Je le sais. Je le remplis. Un carreau garde une trace d'anse.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le métal du toboggan se tait, près du banc. Le seau rentre. Le citron aussi. Le manteau, sur le banc, n'est pas une marche. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est ouvert, comme une rampe douce. On glisse les affaires, sans les jeter. Mila glisse le seau, puis le manteau, puis le citron. Une glissade sage, celle-là. Tu as choisi la pente du sac. Le métal du toboggan se tait, près du sac rouge. Le bol, lui, n'est pas une rampe. Je le sais. Je le remplis. Un carreau garde une trace d'anse.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Le métal du toboggan se tait, près du banc. Le seau rentre. Le citron aussi. Le manteau, sur le banc, n'est pas une marche. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est ouvert, comme une rampe douce. On glisse les affaires, sans les jeter. Mila glisse le seau, puis le manteau, puis le citron. Une glissade sage, celle-là. Merci. Tu as choisi la pente du sac. Le métal du toboggan se tait, près du sac rouge. Le bol, lui, n'est pas une rampe. Je le sais. Je le remplis. Un carreau garde une trace d'anse. [pause]</t>
+          <t>Le métal du toboggan se tait, près du banc. Le seau rentre. Le citron aussi. Le manteau, sur le banc, n'est pas une marche. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est ouvert, comme une rampe douce. On glisse les affaires, sans les jeter. Mila glisse le seau, puis le manteau, puis le citron. Une glissade sage, celle-là. Tu as choisi la pente du sac. Le métal du toboggan se tait, près du sac rouge. Le bol, lui, n'est pas une rampe. Je le sais. Je le remplis. Un carreau garde une trace d'anse. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10223,7 +10210,6 @@
 maman|On glisse les affaires, sans les jeter.
 narrateur|Mila glisse le seau, puis le manteau, puis le citron.
 enfant-f|Une glissade sage, celle-là.
-maman|Merci.
 maman|Tu as choisi la pente du sac.
 narrateur|Le métal du toboggan se tait, près du sac rouge.
 papa|Le bol, lui, n'est pas une rampe.
@@ -10451,17 +10437,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Un pas sur la rampe, derrière. Personne. C'est le vent. On rentre. Seau, manteau, citron. Avant le vent. Le sac à ronds est près de la grille, bouton clair. Tu tournes. Tu glisses. Tu fermes. Mila tourne le bouton. Le seau entre, droit. Le citron, je le tiens jusqu'à la maison. Merci. Tu n'as pas relâché l'anse. Un pas sur la rampe, puis le sac vert se ferme. Le bol n'a pas de vent. Je lui porte son soleil. La virgule verte a un souffle de rampe, on dirait.</t>
+          <t>Un pas sur la rampe, derrière. Personne. C'est le vent. On rentre. Seau, manteau, citron. Avant le vent. Le sac à ronds est près de la grille, bouton clair. Tu tournes. Tu glisses. Tu fermes. Mila tourne le bouton. Le seau entre, droit. Le citron, je le tiens jusqu'à la maison. Tu n'as pas relâché l'anse. Un pas sur la rampe, puis le sac vert se ferme. Le bol n'a pas de vent. Je lui porte son soleil. La virgule verte a un souffle de rampe, on dirait.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un pas sur la rampe, derrière. Personne. C'est le vent. On rentre. Seau, manteau, citron. Avant le vent. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton clair. Tu tournes. Tu glisses. Tu fermes. Mila tourne le bouton. Le seau entre, droit. Le citron, je le tiens jusqu'à la maison. Merci. Tu n'as pas relâché l'anse. Un pas sur la rampe, puis le sac vert se ferme. Le bol n'a pas de vent. Je lui porte son soleil. La virgule verte a un souffle de rampe, on dirait.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un pas sur la rampe, derrière. Personne. C'est le vent. On rentre. Seau, manteau, citron. Avant le vent. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton clair. Tu tournes. Tu glisses. Tu fermes. Mila tourne le bouton. Le seau entre, droit. Le citron, je le tiens jusqu'à la maison. Tu n'as pas relâché l'anse. Un pas sur la rampe, puis le sac vert se ferme. Le bol n'a pas de vent. Je lui porte son soleil. La virgule verte a un souffle de rampe, on dirait.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Un pas sur la rampe, derrière. Personne. C'est le vent. On rentre. Seau, manteau, citron. Avant le vent. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton clair. Tu tournes. Tu glisses. Tu fermes. Mila tourne le bouton. Le seau entre, droit. Le citron, je le tiens jusqu'à la maison. Merci. Tu n'as pas relâché l'anse. Un pas sur la rampe, puis le sac vert se ferme. Le bol n'a pas de vent. Je lui porte son soleil. La virgule verte a un souffle de rampe, on dirait. [pause]</t>
+          <t>Un pas sur la rampe, derrière. Personne. C'est le vent. On rentre. Seau, manteau, citron. Avant le vent. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton clair. Tu tournes. Tu glisses. Tu fermes. Mila tourne le bouton. Le seau entre, droit. Le citron, je le tiens jusqu'à la maison. Tu n'as pas relâché l'anse. Un pas sur la rampe, puis le sac vert se ferme. Le bol n'a pas de vent. Je lui porte son soleil. La virgule verte a un souffle de rampe, on dirait. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10608,7 +10594,6 @@
 narrateur|Mila tourne le bouton.
 narrateur|Le seau entre, droit.
 enfant-f|Le citron, je le tiens jusqu'à la maison.
-papa|Merci.
 papa|Tu n'as pas relâché l'anse.
 narrateur|Un pas sur la rampe, puis le sac vert se ferme.
 maman|Le bol n'a pas de vent.
@@ -11229,17 +11214,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a vu le toboggan, tout gris. On rentre. Le soleil est dans le foulard, plus. Il est dans ta main, maintenant. Le seau aussi. Le sac à étoiles pend. Mila ouvre, le doudou d'abord. Tête vers le zip, pour qu'il respire. Manteau. Seau. Citron contre l'oreille, à vue. Plus de poche. Plus de cachette. Merci. Tu as dénoué le foulard, tout à l'heure. Le doudou a vu le toboggan, dans le sac bleu. Le bol va voir un soleil, lui. Sans foulard. Un fil du foulard reste au zip.</t>
+          <t>Le doudou a vu le toboggan, tout gris. On rentre. Le soleil est dans le foulard, plus. Il est dans ta main, maintenant. Le seau aussi. Le sac à étoiles pend. Mila ouvre, le doudou d'abord. Tête vers le zip, pour qu'il respire. Manteau. Seau. Citron contre l'oreille, à vue. Plus de poche. Plus de cachette. Tu as dénoué le foulard, tout à l'heure. Le doudou a vu le toboggan, dans le sac bleu. Le bol va voir un soleil, lui. Sans foulard. Un fil du foulard reste au zip.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou a vu le toboggan, tout gris. On rentre. Le soleil est dans le foulard, plus. Il est dans ta main, maintenant. Le seau aussi. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila ouvre, le doudou d'abord. Tête vers le zip, pour qu'il respire. Manteau. Seau. Citron contre l'oreille, à vue. Plus de poche. Plus de cachette. Merci. Tu as dénoué le foulard, tout à l'heure. Le doudou a vu le toboggan, dans le sac bleu. Le bol va voir un soleil, lui. Sans foulard. Un fil du foulard reste au zip.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou a vu le toboggan, tout gris. On rentre. Le soleil est dans le foulard, plus. Il est dans ta main, maintenant. Le seau aussi. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila ouvre, le doudou d'abord. Tête vers le zip, pour qu'il respire. Manteau. Seau. Citron contre l'oreille, à vue. Plus de poche. Plus de cachette. Tu as dénoué le foulard, tout à l'heure. Le doudou a vu le toboggan, dans le sac bleu. Le bol va voir un soleil, lui. Sans foulard. Un fil du foulard reste au zip.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a vu le toboggan, tout gris. On rentre. Le soleil est dans le foulard, plus. Il est dans ta main, maintenant. Le seau aussi. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila ouvre, le doudou d'abord. Tête vers le zip, pour qu'il respire. Manteau. Seau. Citron contre l'oreille, à vue. Plus de poche. Plus de cachette. Merci. Tu as dénoué le foulard, tout à l'heure. Le doudou a vu le toboggan, dans le sac bleu. Le bol va voir un soleil, lui. Sans foulard. Un fil du foulard reste au zip. [pause]</t>
+          <t>Le doudou a vu le toboggan, tout gris. On rentre. Le soleil est dans le foulard, plus. Il est dans ta main, maintenant. Le seau aussi. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila ouvre, le doudou d'abord. Tête vers le zip, pour qu'il respire. Manteau. Seau. Citron contre l'oreille, à vue. Plus de poche. Plus de cachette. Tu as dénoué le foulard, tout à l'heure. Le doudou a vu le toboggan, dans le sac bleu. Le bol va voir un soleil, lui. Sans foulard. Un fil du foulard reste au zip. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11386,7 +11371,6 @@
 narrateur|Citron contre l'oreille, à vue.
 enfant-f|Plus de poche.
 enfant-f|Plus de cachette.
-papa|Merci.
 papa|Tu as dénoué le foulard, tout à l'heure.
 narrateur|Le doudou a vu le toboggan, dans le sac bleu.
 maman|Le bol va voir un soleil, lui.
@@ -11613,17 +11597,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>L'oreille molle dépasse, près de la rampe. On a fini de glisser, doudou. Le banc. Le seau. Le manteau. Le sac à carreaux est sur le banc, un carreau plié. Doudou sur le gris du sac. Citron à côté, pas dessous. Mila range. Elle ne recouvre plus le jaune. Je te vois, soleil. Merci. Tu as laissé la virgule à l'air. L'oreille molle dépasse du sac rouge. Le bol, au salon, laissera la feuille à l'air, trop. Oui. Pour la reconnaître. Un carreau garde une odeur de métal.</t>
+          <t>L'oreille molle dépasse, près de la rampe. On a fini de glisser, doudou. Le banc. Le seau. Le manteau. Le sac à carreaux est sur le banc, un carreau plié. Doudou sur le gris du sac. Citron à côté, pas dessous. Mila range. Elle ne recouvre plus le jaune. Je te vois, soleil. Tu as laissé la virgule à l'air. L'oreille molle dépasse du sac rouge. Le bol, au salon, laissera la feuille à l'air, trop. Oui. Pour la reconnaître. Un carreau garde une odeur de métal.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'oreille molle dépasse, près de la rampe. On a fini de glisser, doudou. Le banc. Le seau. Le manteau. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau plié. Doudou sur le gris du sac. Citron à côté, pas dessous. Mila range. Elle ne recouvre plus le jaune. Je te vois, soleil. Merci. Tu as laissé la virgule à l'air. L'oreille molle dépasse du sac rouge. Le bol, au salon, laissera la feuille à l'air, trop. Oui. Pour la reconnaître. Un carreau garde une odeur de métal.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'oreille molle dépasse, près de la rampe. On a fini de glisser, doudou. Le banc. Le seau. Le manteau. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau plié. Doudou sur le gris du sac. Citron à côté, pas dessous. Mila range. Elle ne recouvre plus le jaune. Je te vois, soleil. Tu as laissé la virgule à l'air. L'oreille molle dépasse du sac rouge. Le bol, au salon, laissera la feuille à l'air, trop. Oui. Pour la reconnaître. Un carreau garde une odeur de métal.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>L'oreille molle dépasse, près de la rampe. On a fini de glisser, doudou. Le banc. Le seau. Le manteau. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau plié. Doudou sur le gris du sac. Citron à côté, pas dessous. Mila range. Elle ne recouvre plus le jaune. Je te vois, soleil. Merci. Tu as laissé la virgule à l'air. L'oreille molle dépasse du sac rouge. Le bol, au salon, laissera la feuille à l'air, trop. Oui. Pour la reconnaître. Un carreau garde une odeur de métal. [pause]</t>
+          <t>L'oreille molle dépasse, près de la rampe. On a fini de glisser, doudou. Le banc. Le seau. Le manteau. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau plié. Doudou sur le gris du sac. Citron à côté, pas dessous. Mila range. Elle ne recouvre plus le jaune. Je te vois, soleil. Tu as laissé la virgule à l'air. L'oreille molle dépasse du sac rouge. Le bol, au salon, laissera la feuille à l'air, trop. Oui. Pour la reconnaître. Un carreau garde une odeur de métal. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11768,7 +11752,6 @@
 narrateur|Mila range.
 narrateur|Elle ne recouvre plus le jaune.
 enfant-f|Je te vois, soleil.
-maman|Merci.
 maman|Tu as laissé la virgule à l'air.
 narrateur|L'oreille molle dépasse du sac rouge.
 papa|Le bol, au salon, laissera la feuille à l'air, trop.
@@ -11996,17 +11979,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>La rampe brille. Le doudou cligne, on dirait. On n'y remet pas le jaune. On le met dans le sac à ronds, près de la grille. Le bouton de bois. Mila le tourne, deux fois. Rond le doudou, rond le citron, rond le bouton. Elle glisse le seau, le manteau, le gris, le jaune. Tous visibles, dans la bouche du sac. Merci. Tu n'as rien caché sous le foulard. La rampe brille, loin du sac vert. Le bol n'a pas de rampe. Je le remplis. La virgule verte a une poussière de métal.</t>
+          <t>La rampe brille. Le doudou cligne, on dirait. On n'y remet pas le jaune. On le met dans le sac à ronds, près de la grille. Le bouton de bois. Mila le tourne, deux fois. Rond le doudou, rond le citron, rond le bouton. Elle glisse le seau, le manteau, le gris, le jaune. Tous visibles, dans la bouche du sac. Tu n'as rien caché sous le foulard. La rampe brille, loin du sac vert. Le bol n'a pas de rampe. Je le remplis. La virgule verte a une poussière de métal.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La rampe brille. Le doudou cligne, on dirait. On n'y remet pas le jaune. On le met dans le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt;, près de la grille. Le bouton de bois. Mila le tourne, deux fois. Rond le doudou, rond le citron, rond le bouton. Elle glisse le seau, le manteau, le gris, le jaune. Tous visibles, dans la bouche du sac. Merci. Tu n'as rien caché sous le foulard. La rampe brille, loin du sac vert. Le bol n'a pas de rampe. Je le remplis. La virgule verte a une poussière de métal.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La rampe brille. Le doudou cligne, on dirait. On n'y remet pas le jaune. On le met dans le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt;, près de la grille. Le bouton de bois. Mila le tourne, deux fois. Rond le doudou, rond le citron, rond le bouton. Elle glisse le seau, le manteau, le gris, le jaune. Tous visibles, dans la bouche du sac. Tu n'as rien caché sous le foulard. La rampe brille, loin du sac vert. Le bol n'a pas de rampe. Je le remplis. La virgule verte a une poussière de métal.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>La rampe brille. Le doudou cligne, on dirait. On n'y remet pas le jaune. On le met dans le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt;, près de la grille. Le bouton de bois. Mila le tourne, deux fois. Rond le doudou, rond le citron, rond le bouton. Elle glisse le seau, le manteau, le gris, le jaune. Tous visibles, dans la bouche du sac. Merci. Tu n'as rien caché sous le foulard. La rampe brille, loin du sac vert. Le bol n'a pas de rampe. Je le remplis. La virgule verte a une poussière de métal. [pause]</t>
+          <t>La rampe brille. Le doudou cligne, on dirait. On n'y remet pas le jaune. On le met dans le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt;, près de la grille. Le bouton de bois. Mila le tourne, deux fois. Rond le doudou, rond le citron, rond le bouton. Elle glisse le seau, le manteau, le gris, le jaune. Tous visibles, dans la bouche du sac. Tu n'as rien caché sous le foulard. La rampe brille, loin du sac vert. Le bol n'a pas de rampe. Je le remplis. La virgule verte a une poussière de métal. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -12149,7 +12132,6 @@
 maman|Rond le doudou, rond le citron, rond le bouton.
 narrateur|Elle glisse le seau, le manteau, le gris, le jaune.
 enfant-f|Tous visibles, dans la bouche du sac.
-papa|Merci.
 papa|Tu n'as rien caché sous le foulard.
 narrateur|La rampe brille, loin du sac vert.
 maman|Le bol n'a pas de rampe.
@@ -13536,17 +13518,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Les cordes se taisent. Le ballon penche. J'ai le fil. J'ai le citron. Le seau, au pied de bois, n'a pas de fil. Il vient quand même. Le sac à étoiles pend à la barrière des balançoires. Le zip, et le fil du ballon, c'est pareil un peu. Elle ouvre. Manteau. Seau. Ballon. Citron à l'air. Deux ronds, deux mains, tout à l'heure. Merci. Tu n'as pas relâché le jaune pour le fil. La chaîne a fait cling, près du sac bleu. Le bol n'a pas de fil. Un brin d'herbe reste au cuir, dans le sac.</t>
+          <t>Les cordes se taisent. Le ballon penche. J'ai le fil. J'ai le citron. Le seau, au pied de bois, n'a pas de fil. Il vient quand même. Le sac à étoiles pend à la barrière des balançoires. Le zip, et le fil du ballon, c'est pareil un peu. Elle ouvre. Manteau. Seau. Ballon. Citron à l'air. Deux ronds, deux mains, tout à l'heure. Tu n'as pas relâché le jaune pour le fil. La chaîne a fait cling, près du sac bleu. Le bol n'a pas de fil. Un brin d'herbe reste au cuir, dans le sac.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les cordes se taisent. Le ballon penche. J'ai le fil. J'ai le citron. Le seau, au pied de bois, n'a pas de fil. Il vient quand même. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière des balançoires. Le zip, et le fil du ballon, c'est pareil un peu. Elle ouvre. Manteau. Seau. Ballon. Citron à l'air. Deux ronds, deux mains, tout à l'heure. Merci. Tu n'as pas relâché le jaune pour le fil. La chaîne a fait cling, près du sac bleu. Le bol n'a pas de fil. Un brin d'herbe reste au cuir, dans le sac.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les cordes se taisent. Le ballon penche. J'ai le fil. J'ai le citron. Le seau, au pied de bois, n'a pas de fil. Il vient quand même. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière des balançoires. Le zip, et le fil du ballon, c'est pareil un peu. Elle ouvre. Manteau. Seau. Ballon. Citron à l'air. Deux ronds, deux mains, tout à l'heure. Tu n'as pas relâché le jaune pour le fil. La chaîne a fait cling, près du sac bleu. Le bol n'a pas de fil. Un brin d'herbe reste au cuir, dans le sac.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Les cordes se taisent. Le ballon penche. J'ai le fil. J'ai le citron. Le seau, au pied de bois, n'a pas de fil. Il vient quand même. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière des balançoires. Le zip, et le fil du ballon, c'est pareil un peu. Elle ouvre. Manteau. Seau. Ballon. Citron à l'air. Deux ronds, deux mains, tout à l'heure. Merci. Tu n'as pas relâché le jaune pour le fil. La chaîne a fait cling, près du sac bleu. Le bol n'a pas de fil. Un brin d'herbe reste au cuir, dans le sac. [pause]</t>
+          <t>Les cordes se taisent. Le ballon penche. J'ai le fil. J'ai le citron. Le seau, au pied de bois, n'a pas de fil. Il vient quand même. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend à la barrière des balançoires. Le zip, et le fil du ballon, c'est pareil un peu. Elle ouvre. Manteau. Seau. Ballon. Citron à l'air. Deux ronds, deux mains, tout à l'heure. Tu n'as pas relâché le jaune pour le fil. La chaîne a fait cling, près du sac bleu. Le bol n'a pas de fil. Un brin d'herbe reste au cuir, dans le sac. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13694,7 +13676,6 @@
 narrateur|Ballon.
 narrateur|Citron à l'air.
 maman|Deux ronds, deux mains, tout à l'heure.
-papa|Merci.
 papa|Tu n'as pas relâché le jaune pour le fil.
 narrateur|La chaîne a fait cling, près du sac bleu.
 enfant-f|Le bol n'a pas de fil.
@@ -13921,17 +13902,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Le ballon a touché le sable, près des balançoires. On rentre. Le rouge et le jaune. Le pied de bois a le seau. Le banc a le manteau. Le sac à carreaux est sur le banc des balançoires. Un carreau pour le fil, enroulé. Un carreau pour le jaune. Mila enroule le fil. Elle pose le citron à part. Vous ne vous mélangez plus. Merci. Tu as séparé l'ombre rouge du jaune. Le ballon a touché le sable, près du sac rouge. Le bol n'a pas d'ombre rouge. Que du bleu, et mon soleil. Un carreau garde un brin d'herbe.</t>
+          <t>Le ballon a touché le sable, près des balançoires. On rentre. Le rouge et le jaune. Le pied de bois a le seau. Le banc a le manteau. Le sac à carreaux est sur le banc des balançoires. Un carreau pour le fil, enroulé. Un carreau pour le jaune. Mila enroule le fil. Elle pose le citron à part. Vous ne vous mélangez plus. Tu as séparé l'ombre rouge du jaune. Le ballon a touché le sable, près du sac rouge. Le bol n'a pas d'ombre rouge. Que du bleu, et mon soleil. Un carreau garde un brin d'herbe.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon a touché le sable, près des balançoires. On rentre. Le rouge et le jaune. Le pied de bois a le seau. Le banc a le manteau. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc des balançoires. Un carreau pour le fil, enroulé. Un carreau pour le jaune. Mila enroule le fil. Elle pose le citron à part. Vous ne vous mélangez plus. Merci. Tu as séparé l'ombre rouge du jaune. Le ballon a touché le sable, près du sac rouge. Le bol n'a pas d'ombre rouge. Que du bleu, et mon soleil. Un carreau garde un brin d'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon a touché le sable, près des balançoires. On rentre. Le rouge et le jaune. Le pied de bois a le seau. Le banc a le manteau. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc des balançoires. Un carreau pour le fil, enroulé. Un carreau pour le jaune. Mila enroule le fil. Elle pose le citron à part. Vous ne vous mélangez plus. Tu as séparé l'ombre rouge du jaune. Le ballon a touché le sable, près du sac rouge. Le bol n'a pas d'ombre rouge. Que du bleu, et mon soleil. Un carreau garde un brin d'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Le ballon a touché le sable, près des balançoires. On rentre. Le rouge et le jaune. Le pied de bois a le seau. Le banc a le manteau. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc des balançoires. Un carreau pour le fil, enroulé. Un carreau pour le jaune. Mila enroule le fil. Elle pose le citron à part. Vous ne vous mélangez plus. Merci. Tu as séparé l'ombre rouge du jaune. Le ballon a touché le sable, près du sac rouge. Le bol n'a pas d'ombre rouge. Que du bleu, et mon soleil. Un carreau garde un brin d'herbe. [pause]</t>
+          <t>Le ballon a touché le sable, près des balançoires. On rentre. Le rouge et le jaune. Le pied de bois a le seau. Le banc a le manteau. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc des balançoires. Un carreau pour le fil, enroulé. Un carreau pour le jaune. Mila enroule le fil. Elle pose le citron à part. Vous ne vous mélangez plus. Tu as séparé l'ombre rouge du jaune. Le ballon a touché le sable, près du sac rouge. Le bol n'a pas d'ombre rouge. Que du bleu, et mon soleil. Un carreau garde un brin d'herbe. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -14076,7 +14057,6 @@
 narrateur|Mila enroule le fil.
 narrateur|Elle pose le citron à part.
 enfant-f|Vous ne vous mélangez plus.
-maman|Merci.
 maman|Tu as séparé l'ombre rouge du jaune.
 narrateur|Le ballon a touché le sable, près du sac rouge.
 papa|Le bol n'a pas d'ombre rouge.
@@ -14302,17 +14282,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Un nuage passe au-dessus des balançoires. Le ballon baisse. On rentre. Seau, manteau, citron. Avant que le nuage reste. Le sac à ronds est près de la grille, bouton pâle. Tu tournes. Tu comptes les ronds. Ballon. Citron. Bouton. Seau. Manteau. Cinq. Tous là. Merci. Tu as compté le jaune, pas seulement le rouge. Un nuage passe au-dessus du sac vert. Le bol, sous le toit, n'a pas de nuage. Il a un rond de lumière. La virgule verte a une ombre de nuage, un instant.</t>
+          <t>Un nuage passe au-dessus des balançoires. Le ballon baisse. On rentre. Seau, manteau, citron. Avant que le nuage reste. Le sac à ronds est près de la grille, bouton pâle. Tu tournes. Tu comptes les ronds. Ballon. Citron. Bouton. Seau. Manteau. Cinq. Tous là. Tu as compté le jaune, pas seulement le rouge. Un nuage passe au-dessus du sac vert. Le bol, sous le toit, n'a pas de nuage. Il a un rond de lumière. La virgule verte a une ombre de nuage, un instant.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un nuage passe au-dessus des balançoires. Le ballon baisse. On rentre. Seau, manteau, citron. Avant que le nuage reste. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton pâle. Tu tournes. Tu comptes les ronds. Ballon. Citron. Bouton. Seau. Manteau. Cinq. Tous là. Merci. Tu as compté le jaune, pas seulement le rouge. Un nuage passe au-dessus du sac vert. Le bol, sous le toit, n'a pas de nuage. Il a un rond de lumière. La virgule verte a une ombre de nuage, un instant.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un nuage passe au-dessus des balançoires. Le ballon baisse. On rentre. Seau, manteau, citron. Avant que le nuage reste. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton pâle. Tu tournes. Tu comptes les ronds. Ballon. Citron. Bouton. Seau. Manteau. Cinq. Tous là. Tu as compté le jaune, pas seulement le rouge. Un nuage passe au-dessus du sac vert. Le bol, sous le toit, n'a pas de nuage. Il a un rond de lumière. La virgule verte a une ombre de nuage, un instant.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Un nuage passe au-dessus des balançoires. Le ballon baisse. On rentre. Seau, manteau, citron. Avant que le nuage reste. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton pâle. Tu tournes. Tu comptes les ronds. Ballon. Citron. Bouton. Seau. Manteau. Cinq. Tous là. Merci. Tu as compté le jaune, pas seulement le rouge. Un nuage passe au-dessus du sac vert. Le bol, sous le toit, n'a pas de nuage. Il a un rond de lumière. La virgule verte a une ombre de nuage, un instant. [pause]</t>
+          <t>Un nuage passe au-dessus des balançoires. Le ballon baisse. On rentre. Seau, manteau, citron. Avant que le nuage reste. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton pâle. Tu tournes. Tu comptes les ronds. Ballon. Citron. Bouton. Seau. Manteau. Cinq. Tous là. Tu as compté le jaune, pas seulement le rouge. Un nuage passe au-dessus du sac vert. Le bol, sous le toit, n'a pas de nuage. Il a un rond de lumière. La virgule verte a une ombre de nuage, un instant. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14461,7 +14441,6 @@
 narrateur|Manteau.
 enfant-f|Cinq.
 enfant-f|Tous là.
-papa|Merci.
 papa|Tu as compté le jaune, pas seulement le rouge.
 narrateur|Un nuage passe au-dessus du sac vert.
 maman|Le bol, sous le toit, n'a pas de nuage.
@@ -15081,17 +15060,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Le seau a servi de nid, sous la balançoire. On rentre. Le nid vient. Le banc a le manteau. Il n'est pas un nid. Le sac à étoiles pend. Mila hisse le seau. L'anse, deux mains, comme tout à l'heure. Le seau entre. Le manteau. Le citron au fond, à vue. Un nid qui voyage, pour le bol. Merci. Tes tibias ont ramené le seau. L'anse du seau est froide, contre le sac bleu. Le bol n'a pas d'anse. Je connais son bord. Une étoile de tissu a une trace d'herbe.</t>
+          <t>Le seau a servi de nid, sous la balançoire. On rentre. Le nid vient. Le banc a le manteau. Il n'est pas un nid. Le sac à étoiles pend. Mila hisse le seau. L'anse, deux mains, comme tout à l'heure. Le seau entre. Le manteau. Le citron au fond, à vue. Un nid qui voyage, pour le bol. Tes tibias ont ramené le seau. L'anse du seau est froide, contre le sac bleu. Le bol n'a pas d'anse. Je connais son bord. Une étoile de tissu a une trace d'herbe.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau a servi de nid, sous la balançoire. On rentre. Le nid vient. Le banc a le manteau. Il n'est pas un nid. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila hisse le seau. L'anse, deux mains, comme tout à l'heure. Le seau entre. Le manteau. Le citron au fond, à vue. Un nid qui voyage, pour le bol. Merci. Tes tibias ont ramené le seau. L'anse du seau est froide, contre le sac bleu. Le bol n'a pas d'anse. Je connais son bord. Une étoile de tissu a une trace d'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau a servi de nid, sous la balançoire. On rentre. Le nid vient. Le banc a le manteau. Il n'est pas un nid. Le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila hisse le seau. L'anse, deux mains, comme tout à l'heure. Le seau entre. Le manteau. Le citron au fond, à vue. Un nid qui voyage, pour le bol. Tes tibias ont ramené le seau. L'anse du seau est froide, contre le sac bleu. Le bol n'a pas d'anse. Je connais son bord. Une étoile de tissu a une trace d'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Le seau a servi de nid, sous la balançoire. On rentre. Le nid vient. Le banc a le manteau. Il n'est pas un nid. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila hisse le seau. L'anse, deux mains, comme tout à l'heure. Le seau entre. Le manteau. Le citron au fond, à vue. Un nid qui voyage, pour le bol. Merci. Tes tibias ont ramené le seau. L'anse du seau est froide, contre le sac bleu. Le bol n'a pas d'anse. Je connais son bord. Une étoile de tissu a une trace d'herbe. [pause]</t>
+          <t>Le seau a servi de nid, sous la balançoire. On rentre. Le nid vient. Le banc a le manteau. Il n'est pas un nid. Le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt; pend. Mila hisse le seau. L'anse, deux mains, comme tout à l'heure. Le seau entre. Le manteau. Le citron au fond, à vue. Un nid qui voyage, pour le bol. Tes tibias ont ramené le seau. L'anse du seau est froide, contre le sac bleu. Le bol n'a pas d'anse. Je connais son bord. Une étoile de tissu a une trace d'herbe. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -15237,7 +15216,6 @@
 narrateur|Le manteau.
 narrateur|Le citron au fond, à vue.
 enfant-f|Un nid qui voyage, pour le bol.
-papa|Merci.
 papa|Tes tibias ont ramené le seau.
 narrateur|L'anse du seau est froide, contre le sac bleu.
 maman|Le bol n'a pas d'anse.
@@ -15464,17 +15442,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Un cling lointain. Une autre balançoire, loin. La nôtre s'est arrêtée. On rentre. Nid, manteau, citron. Avant le cling des autres. Le sac à carreaux est sur le banc, un carreau ouvert. Le seau sur le carreau du bas. Le citron sur le clair. Mila range. Elle ne met plus le seau sous ses pieds. Le nid, dans le sac. Pas sous les talons. Merci. Tu as changé la place du seau. Un cling lointain, et le sac rouge se ferme. Le bol n'a pas de cling. Je le lui rends, le clic. Un carreau garde une trace de tibia, de poussière.</t>
+          <t>Un cling lointain. Une autre balançoire, loin. La nôtre s'est arrêtée. On rentre. Nid, manteau, citron. Avant le cling des autres. Le sac à carreaux est sur le banc, un carreau ouvert. Le seau sur le carreau du bas. Le citron sur le clair. Mila range. Elle ne met plus le seau sous ses pieds. Le nid, dans le sac. Pas sous les talons. Tu as changé la place du seau. Un cling lointain, et le sac rouge se ferme. Le bol n'a pas de cling. Je le lui rends, le clic. Un carreau garde une trace de tibia, de poussière.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un cling lointain. Une autre balançoire, loin. La nôtre s'est arrêtée. On rentre. Nid, manteau, citron. Avant le cling des autres. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau ouvert. Le seau sur le carreau du bas. Le citron sur le clair. Mila range. Elle ne met plus le seau sous ses pieds. Le nid, dans le sac. Pas sous les talons. Merci. Tu as changé la place du seau. Un cling lointain, et le sac rouge se ferme. Le bol n'a pas de cling. Je le lui rends, le clic. Un carreau garde une trace de tibia, de poussière.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un cling lointain. Une autre balançoire, loin. La nôtre s'est arrêtée. On rentre. Nid, manteau, citron. Avant le cling des autres. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau ouvert. Le seau sur le carreau du bas. Le citron sur le clair. Mila range. Elle ne met plus le seau sous ses pieds. Le nid, dans le sac. Pas sous les talons. Tu as changé la place du seau. Un cling lointain, et le sac rouge se ferme. Le bol n'a pas de cling. Je le lui rends, le clic. Un carreau garde une trace de tibia, de poussière.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Un cling lointain. Une autre balançoire, loin. La nôtre s'est arrêtée. On rentre. Nid, manteau, citron. Avant le cling des autres. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau ouvert. Le seau sur le carreau du bas. Le citron sur le clair. Mila range. Elle ne met plus le seau sous ses pieds. Le nid, dans le sac. Pas sous les talons. Merci. Tu as changé la place du seau. Un cling lointain, et le sac rouge se ferme. Le bol n'a pas de cling. Je le lui rends, le clic. Un carreau garde une trace de tibia, de poussière. [pause]</t>
+          <t>Un cling lointain. Une autre balançoire, loin. La nôtre s'est arrêtée. On rentre. Nid, manteau, citron. Avant le cling des autres. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau ouvert. Le seau sur le carreau du bas. Le citron sur le clair. Mila range. Elle ne met plus le seau sous ses pieds. Le nid, dans le sac. Pas sous les talons. Tu as changé la place du seau. Un cling lointain, et le sac rouge se ferme. Le bol n'a pas de cling. Je le lui rends, le clic. Un carreau garde une trace de tibia, de poussière. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15621,7 +15599,6 @@
 narrateur|Elle ne met plus le seau sous ses pieds.
 enfant-f|Le nid, dans le sac.
 enfant-f|Pas sous les talons.
-maman|Merci.
 maman|Tu as changé la place du seau.
 narrateur|Un cling lointain, et le sac rouge se ferme.
 papa|Le bol n'a pas de cling.
@@ -15847,17 +15824,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le seau jaune pose son ombre au pied de bois. L'ombre rentre, elle aussi. Le manteau. Le seau. Le citron. Le sac à ronds est près de la grille, bouton rond. L'ombre du seau, ronde, rentre dans un rond. Mila glisse le seau, le manteau, le citron au milieu. Le nid au milieu, comme sous la balançoire. Mais fermé. Merci. Tu as fermé le nid, cette fois. Le seau jaune pose son ombre au sac vert. Le bol a un rond de lumière, pas d'ombre de seau. Je lui donne le soleil, pas l'ombre. La virgule verte a une poussière de pied de bois.</t>
+          <t>Le seau jaune pose son ombre au pied de bois. L'ombre rentre, elle aussi. Le manteau. Le seau. Le citron. Le sac à ronds est près de la grille, bouton rond. L'ombre du seau, ronde, rentre dans un rond. Mila glisse le seau, le manteau, le citron au milieu. Le nid au milieu, comme sous la balançoire. Mais fermé. Tu as fermé le nid, cette fois. Le seau jaune pose son ombre au sac vert. Le bol a un rond de lumière, pas d'ombre de seau. Je lui donne le soleil, pas l'ombre. La virgule verte a une poussière de pied de bois.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau jaune pose son ombre au pied de bois. L'ombre rentre, elle aussi. Le manteau. Le seau. Le citron. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton rond. L'ombre du seau, ronde, rentre dans un rond. Mila glisse le seau, le manteau, le citron au milieu. Le nid au milieu, comme sous la balançoire. Mais fermé. Merci. Tu as fermé le nid, cette fois. Le seau jaune pose son ombre au sac vert. Le bol a un rond de lumière, pas d'ombre de seau. Je lui donne le soleil, pas l'ombre. La virgule verte a une poussière de pied de bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau jaune pose son ombre au pied de bois. L'ombre rentre, elle aussi. Le manteau. Le seau. Le citron. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton rond. L'ombre du seau, ronde, rentre dans un rond. Mila glisse le seau, le manteau, le citron au milieu. Le nid au milieu, comme sous la balançoire. Mais fermé. Tu as fermé le nid, cette fois. Le seau jaune pose son ombre au sac vert. Le bol a un rond de lumière, pas d'ombre de seau. Je lui donne le soleil, pas l'ombre. La virgule verte a une poussière de pied de bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Le seau jaune pose son ombre au pied de bois. L'ombre rentre, elle aussi. Le manteau. Le seau. Le citron. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton rond. L'ombre du seau, ronde, rentre dans un rond. Mila glisse le seau, le manteau, le citron au milieu. Le nid au milieu, comme sous la balançoire. Mais fermé. Merci. Tu as fermé le nid, cette fois. Le seau jaune pose son ombre au sac vert. Le bol a un rond de lumière, pas d'ombre de seau. Je lui donne le soleil, pas l'ombre. La virgule verte a une poussière de pied de bois. [pause]</t>
+          <t>Le seau jaune pose son ombre au pied de bois. L'ombre rentre, elle aussi. Le manteau. Le seau. Le citron. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt; est près de la grille, bouton rond. L'ombre du seau, ronde, rentre dans un rond. Mila glisse le seau, le manteau, le citron au milieu. Le nid au milieu, comme sous la balançoire. Mais fermé. Tu as fermé le nid, cette fois. Le seau jaune pose son ombre au sac vert. Le bol a un rond de lumière, pas d'ombre de seau. Je lui donne le soleil, pas l'ombre. La virgule verte a une poussière de pied de bois. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -16001,7 +15978,6 @@
 narrateur|Mila glisse le seau, le manteau, le citron au milieu.
 enfant-f|Le nid au milieu, comme sous la balançoire.
 enfant-f|Mais fermé.
-papa|Merci.
 papa|Tu as fermé le nid, cette fois.
 narrateur|Le seau jaune pose son ombre au sac vert.
 maman|Le bol a un rond de lumière, pas d'ombre de seau.
@@ -16621,17 +16597,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a senti le vent, entre les sièges. On ne se passe plus le soleil en l'air. On le passe dans le sac à étoiles, à la barrière. Mila ouvre le zip. Le doudou entre, assis. Le citron à côté, pas entre les sièges. Seau. Manteau. Jaune à vue, contre le gris. Les mains, pas l'air. Merci. Tu as cherché la virgule, pas la colère. Le doudou a senti le vent, dans le sac bleu. Le bol n'a pas de vent. Je lui porte le soleil, dans les mains. Un fil gris pend, pris dans une étoile.</t>
+          <t>Le doudou a senti le vent, entre les sièges. On ne se passe plus le soleil en l'air. On le passe dans le sac à étoiles, à la barrière. Mila ouvre le zip. Le doudou entre, assis. Le citron à côté, pas entre les sièges. Seau. Manteau. Jaune à vue, contre le gris. Les mains, pas l'air. Tu as cherché la virgule, pas la colère. Le doudou a senti le vent, dans le sac bleu. Le bol n'a pas de vent. Je lui porte le soleil, dans les mains. Un fil gris pend, pris dans une étoile.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou a senti le vent, entre les sièges. On ne se passe plus le soleil en l'air. On le passe dans le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt;, à la barrière. Mila ouvre le zip. Le doudou entre, assis. Le citron à côté, pas entre les sièges. Seau. Manteau. Jaune à vue, contre le gris. Les mains, pas l'air. Merci. Tu as cherché la virgule, pas la colère. Le doudou a senti le vent, dans le sac bleu. Le bol n'a pas de vent. Je lui porte le soleil, dans les mains. Un fil gris pend, pris dans une étoile.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou a senti le vent, entre les sièges. On ne se passe plus le soleil en l'air. On le passe dans le &lt;emphasis level="moderate"&gt;sac à étoiles&lt;/emphasis&gt;, à la barrière. Mila ouvre le zip. Le doudou entre, assis. Le citron à côté, pas entre les sièges. Seau. Manteau. Jaune à vue, contre le gris. Les mains, pas l'air. Tu as cherché la virgule, pas la colère. Le doudou a senti le vent, dans le sac bleu. Le bol n'a pas de vent. Je lui porte le soleil, dans les mains. Un fil gris pend, pris dans une étoile.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a senti le vent, entre les sièges. On ne se passe plus le soleil en l'air. On le passe dans le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt;, à la barrière. Mila ouvre le zip. Le doudou entre, assis. Le citron à côté, pas entre les sièges. Seau. Manteau. Jaune à vue, contre le gris. Les mains, pas l'air. Merci. Tu as cherché la virgule, pas la colère. Le doudou a senti le vent, dans le sac bleu. Le bol n'a pas de vent. Je lui porte le soleil, dans les mains. Un fil gris pend, pris dans une étoile. [pause]</t>
+          <t>Le doudou a senti le vent, entre les sièges. On ne se passe plus le soleil en l'air. On le passe dans le &lt;emphasis&gt;sac à étoiles&lt;/emphasis&gt;, à la barrière. Mila ouvre le zip. Le doudou entre, assis. Le citron à côté, pas entre les sièges. Seau. Manteau. Jaune à vue, contre le gris. Les mains, pas l'air. Tu as cherché la virgule, pas la colère. Le doudou a senti le vent, dans le sac bleu. Le bol n'a pas de vent. Je lui porte le soleil, dans les mains. Un fil gris pend, pris dans une étoile. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16775,7 +16751,6 @@
 narrateur|Manteau.
 narrateur|Jaune à vue, contre le gris.
 enfant-f|Les mains, pas l'air.
-papa|Merci.
 papa|Tu as cherché la virgule, pas la colère.
 narrateur|Le doudou a senti le vent, dans le sac bleu.
 maman|Le bol n'a pas de vent.
@@ -17001,17 +16976,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>La chaîne se tait, près du banc. Le doudou rentre. Le citron aussi. Le seau au pied. Le manteau au banc. Le sac à carreaux est sur le banc, un carreau pour le gris. Doudou. Seau. Manteau. Citron à part, visible. Mila ne lance plus. Elle pose. Posé, pas lancé. Merci. Tes mains ont appris le passage. La chaîne se tait, près du sac rouge. Le bol n'a pas de chaîne. Je pose, sur le bord. Un carreau garde une poussière de siège.</t>
+          <t>La chaîne se tait, près du banc. Le doudou rentre. Le citron aussi. Le seau au pied. Le manteau au banc. Le sac à carreaux est sur le banc, un carreau pour le gris. Doudou. Seau. Manteau. Citron à part, visible. Mila ne lance plus. Elle pose. Posé, pas lancé. Tes mains ont appris le passage. La chaîne se tait, près du sac rouge. Le bol n'a pas de chaîne. Je pose, sur le bord. Un carreau garde une poussière de siège.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La chaîne se tait, près du banc. Le doudou rentre. Le citron aussi. Le seau au pied. Le manteau au banc. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau pour le gris. Doudou. Seau. Manteau. Citron à part, visible. Mila ne lance plus. Elle pose. Posé, pas lancé. Merci. Tes mains ont appris le passage. La chaîne se tait, près du sac rouge. Le bol n'a pas de chaîne. Je pose, sur le bord. Un carreau garde une poussière de siège.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La chaîne se tait, près du banc. Le doudou rentre. Le citron aussi. Le seau au pied. Le manteau au banc. Le &lt;emphasis level="moderate"&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau pour le gris. Doudou. Seau. Manteau. Citron à part, visible. Mila ne lance plus. Elle pose. Posé, pas lancé. Tes mains ont appris le passage. La chaîne se tait, près du sac rouge. Le bol n'a pas de chaîne. Je pose, sur le bord. Un carreau garde une poussière de siège.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>La chaîne se tait, près du banc. Le doudou rentre. Le citron aussi. Le seau au pied. Le manteau au banc. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau pour le gris. Doudou. Seau. Manteau. Citron à part, visible. Mila ne lance plus. Elle pose. Posé, pas lancé. Merci. Tes mains ont appris le passage. La chaîne se tait, près du sac rouge. Le bol n'a pas de chaîne. Je pose, sur le bord. Un carreau garde une poussière de siège. [pause]</t>
+          <t>La chaîne se tait, près du banc. Le doudou rentre. Le citron aussi. Le seau au pied. Le manteau au banc. Le &lt;emphasis&gt;sac à carreaux&lt;/emphasis&gt; est sur le banc, un carreau pour le gris. Doudou. Seau. Manteau. Citron à part, visible. Mila ne lance plus. Elle pose. Posé, pas lancé. Tes mains ont appris le passage. La chaîne se tait, près du sac rouge. Le bol n'a pas de chaîne. Je pose, sur le bord. Un carreau garde une poussière de siège. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -17158,7 +17133,6 @@
 narrateur|Mila ne lance plus.
 narrateur|Elle pose.
 enfant-f|Posé, pas lancé.
-maman|Merci.
 maman|Tes mains ont appris le passage.
 narrateur|La chaîne se tait, près du sac rouge.
 papa|Le bol n'a pas de chaîne.
@@ -17386,17 +17360,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>L'oreille grise dépasse, entre les deux sièges vides. On rentre. Le vent peut garder les cordes. Le sac à ronds, près de la grille, garde le reste. Mila tourne le bouton. Ça cède. Rond l'oreille, rond le citron, rond le bouton. Elle glisse le doudou, le seau, le manteau, le jaune. Le campement du salon va tout revoir. Merci. Tu as ramassé entre les pieds de bois. L'oreille grise dépasse du sac vert. Le bol a un rond de lumière, qui t'attend. Je lui rends son soleil. La virgule verte a de la poussière, et de l'herbe.</t>
+          <t>L'oreille grise dépasse, entre les deux sièges vides. On rentre. Le vent peut garder les cordes. Le sac à ronds, près de la grille, garde le reste. Mila tourne le bouton. Ça cède. Rond l'oreille, rond le citron, rond le bouton. Elle glisse le doudou, le seau, le manteau, le jaune. Le campement du salon va tout revoir. Tu as ramassé entre les pieds de bois. L'oreille grise dépasse du sac vert. Le bol a un rond de lumière, qui t'attend. Je lui rends son soleil. La virgule verte a de la poussière, et de l'herbe.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'oreille grise dépasse, entre les deux sièges vides. On rentre. Le vent peut garder les cordes. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt;, près de la grille, garde le reste. Mila tourne le bouton. Ça cède. Rond l'oreille, rond le citron, rond le bouton. Elle glisse le doudou, le seau, le manteau, le jaune. Le campement du salon va tout revoir. Merci. Tu as ramassé entre les pieds de bois. L'oreille grise dépasse du sac vert. Le bol a un rond de lumière, qui t'attend. Je lui rends son soleil. La virgule verte a de la poussière, et de l'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'oreille grise dépasse, entre les deux sièges vides. On rentre. Le vent peut garder les cordes. Le &lt;emphasis level="moderate"&gt;sac à ronds&lt;/emphasis&gt;, près de la grille, garde le reste. Mila tourne le bouton. Ça cède. Rond l'oreille, rond le citron, rond le bouton. Elle glisse le doudou, le seau, le manteau, le jaune. Le campement du salon va tout revoir. Tu as ramassé entre les pieds de bois. L'oreille grise dépasse du sac vert. Le bol a un rond de lumière, qui t'attend. Je lui rends son soleil. La virgule verte a de la poussière, et de l'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>L'oreille grise dépasse, entre les deux sièges vides. On rentre. Le vent peut garder les cordes. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt;, près de la grille, garde le reste. Mila tourne le bouton. Ça cède. Rond l'oreille, rond le citron, rond le bouton. Elle glisse le doudou, le seau, le manteau, le jaune. Le campement du salon va tout revoir. Merci. Tu as ramassé entre les pieds de bois. L'oreille grise dépasse du sac vert. Le bol a un rond de lumière, qui t'attend. Je lui rends son soleil. La virgule verte a de la poussière, et de l'herbe. [pause]</t>
+          <t>L'oreille grise dépasse, entre les deux sièges vides. On rentre. Le vent peut garder les cordes. Le &lt;emphasis&gt;sac à ronds&lt;/emphasis&gt;, près de la grille, garde le reste. Mila tourne le bouton. Ça cède. Rond l'oreille, rond le citron, rond le bouton. Elle glisse le doudou, le seau, le manteau, le jaune. Le campement du salon va tout revoir. Tu as ramassé entre les pieds de bois. L'oreille grise dépasse du sac vert. Le bol a un rond de lumière, qui t'attend. Je lui rends son soleil. La virgule verte a de la poussière, et de l'herbe. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17539,7 +17513,6 @@
 maman|Rond l'oreille, rond le citron, rond le bouton.
 narrateur|Elle glisse le doudou, le seau, le manteau, le jaune.
 enfant-f|Le campement du salon va tout revoir.
-papa|Merci.
 papa|Tu as ramassé entre les pieds de bois.
 narrateur|L'oreille grise dépasse du sac vert.
 maman|Le bol a un rond de lumière, qui t'attend.
@@ -17761,7 +17734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17874,6 +17847,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>